<commit_message>
Enhance data.md with new columns for tracking weekly usage pace and historical context. Update index.html to improve user guidance on product switching and boost values, including dynamic calculations for pace and time elapsed. Update binary files for usage tracking visuals.
</commit_message>
<xml_diff>
--- a/Claude_kostnad/Claude_usage.xlsx
+++ b/Claude_kostnad/Claude_usage.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ovrigt/Claude_kostnad/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="8_{47C55551-E54E-40CD-A718-3CAE99F89ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB7035D8-8B8C-4B8D-B8A4-5AB3F4F2DA2E}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="8_{47C55551-E54E-40CD-A718-3CAE99F89ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{636A7915-F16D-4DFE-BEC4-1EC2C84F6700}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FC573CD4-0E63-4713-BCBE-D8AF6B5A970C}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FC573CD4-0E63-4713-BCBE-D8AF6B5A970C}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Thu</t>
   </si>
@@ -85,13 +85,19 @@
   </si>
   <si>
     <t>Hade det varit 41 % av av en vecka kvar till återställning av vecko-tookens hade jag legat precis i fas med med mitt pro-Claude-abonnemang. Trodde jag först…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utveckla </t>
+  </si>
+  <si>
+    <t>https://kentlundgren.github.io/Ovrigt/Claude_kostnad/index.html</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -115,6 +121,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -133,18 +164,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlänk" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -506,55 +541,71 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12FDF2DA-B207-4AB6-8F36-12DE6A1A841A}">
-  <dimension ref="I3:L22"/>
+  <dimension ref="I1:Q22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="9:17" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+    </row>
+    <row r="2" spans="9:17" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="9:17" x14ac:dyDescent="0.25">
       <c r="I3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="9:17" x14ac:dyDescent="0.25">
       <c r="I4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="9:17" x14ac:dyDescent="0.25">
       <c r="I5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="9:17" x14ac:dyDescent="0.25">
       <c r="I6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="9:17" x14ac:dyDescent="0.25">
       <c r="I7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="9:17" x14ac:dyDescent="0.25">
       <c r="I8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="9:17" x14ac:dyDescent="0.25">
       <c r="I9" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="9:17" x14ac:dyDescent="0.25">
       <c r="I10" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="12" spans="9:17" x14ac:dyDescent="0.25">
       <c r="L12" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="13" spans="9:17" x14ac:dyDescent="0.25">
       <c r="I13" t="s">
         <v>2</v>
       </c>
@@ -565,7 +616,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="14" spans="9:17" x14ac:dyDescent="0.25">
       <c r="I14" t="s">
         <v>3</v>
       </c>
@@ -576,7 +627,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="15" spans="9:17" x14ac:dyDescent="0.25">
       <c r="I15" t="s">
         <v>4</v>
       </c>
@@ -587,7 +638,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="9:12" x14ac:dyDescent="0.25">
+    <row r="16" spans="9:17" x14ac:dyDescent="0.25">
       <c r="I16" t="s">
         <v>0</v>
       </c>
@@ -647,7 +698,10 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="J1" r:id="rId1" xr:uid="{3C0910C9-889C-4471-9944-487CEFBFB178}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update data.md with new usage readings and historical context, confirming the overflow mechanism and adjustments in session limits. Modify index.html to reflect updated weekly percentage input and add a new output for purchased credits. Enhance SKILL.md with clarifications on usage credits and billing distinctions. Introduce a new image file for visual representation of usage data.
</commit_message>
<xml_diff>
--- a/Claude_kostnad/Claude_usage.xlsx
+++ b/Claude_kostnad/Claude_usage.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ovrigt/Claude_kostnad/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="8_{47C55551-E54E-40CD-A718-3CAE99F89ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{636A7915-F16D-4DFE-BEC4-1EC2C84F6700}"/>
+  <xr:revisionPtr revIDLastSave="139" documentId="8_{47C55551-E54E-40CD-A718-3CAE99F89ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95672569-80AD-4ADF-9A80-EFA32C806D72}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FC573CD4-0E63-4713-BCBE-D8AF6B5A970C}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FC573CD4-0E63-4713-BCBE-D8AF6B5A970C}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
+    <sheet name="Blad2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
   <si>
     <t>Thu</t>
   </si>
@@ -91,13 +92,25 @@
   </si>
   <si>
     <t>https://kentlundgren.github.io/Ovrigt/Claude_kostnad/index.html</t>
+  </si>
+  <si>
+    <t>Vad jag köpt extra under april månad:</t>
+  </si>
+  <si>
+    <t>EUR</t>
+  </si>
+  <si>
+    <t>Har jag köpt något extra denna månad, i augusti 2026:</t>
+  </si>
+  <si>
+    <t>TOT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -146,6 +159,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -168,15 +197,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlänk" xfId="1" builtinId="8"/>
@@ -233,6 +271,99 @@
         <a:xfrm>
           <a:off x="4838700" y="2047875"/>
           <a:ext cx="9142857" cy="4752381"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>598920</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>113434</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Bildobjekt 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6EF3B2DF-A4DF-79A6-21D7-19BA5228350E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3638550" y="12039600"/>
+          <a:ext cx="9238095" cy="6923809"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>180974</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>75032</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>19049</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Bildobjekt 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D561242E-6A37-3EE5-7026-13243D4FB39B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3619500" y="1971674"/>
+          <a:ext cx="9342857" cy="9553575"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -545,19 +676,19 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="9:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
     </row>
     <row r="2" spans="9:17" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="9:17" x14ac:dyDescent="0.25">
@@ -704,4 +835,105 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C51D97A-C046-4E26-9C29-4DD7EDCC8104}">
+  <dimension ref="F1:I63"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="G1" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="6:9" ht="21" x14ac:dyDescent="0.35">
+      <c r="G3" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="G5" s="7">
+        <v>46125</v>
+      </c>
+      <c r="H5" s="11">
+        <v>6.25</v>
+      </c>
+      <c r="I5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="G6" s="7">
+        <v>46139</v>
+      </c>
+      <c r="H6" s="11">
+        <v>47.81</v>
+      </c>
+      <c r="I6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="G7" s="7">
+        <v>46140</v>
+      </c>
+      <c r="H7" s="11">
+        <v>12.5</v>
+      </c>
+      <c r="I7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F8" s="10"/>
+      <c r="G8" s="7">
+        <v>46122</v>
+      </c>
+      <c r="H8" s="11">
+        <v>12.5</v>
+      </c>
+      <c r="I8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F9" s="10"/>
+      <c r="G9" s="7">
+        <v>46122</v>
+      </c>
+      <c r="H9" s="11">
+        <v>12.5</v>
+      </c>
+      <c r="I9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="G10" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10" s="12">
+        <f>SUM(H5:H9)</f>
+        <v>91.56</v>
+      </c>
+      <c r="I10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="63" spans="7:7" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="G63" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G1" r:id="rId1" xr:uid="{10317F2F-351C-4BF7-AB20-570B457158DA}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add daily consumption tracking routine starting 2026-08-04 in data.md and index.html. Introduced a new table for daily usage credits in euros, updated manually each evening based on Kent's readings. Documented exception for the first day's calculation. Enhanced SKILL.md with details on the new routine and its implementation.
</commit_message>
<xml_diff>
--- a/Claude_kostnad/Claude_usage.xlsx
+++ b/Claude_kostnad/Claude_usage.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4768e0e598e90526/AI/Claude/Ovrigt/Claude_kostnad/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="139" documentId="8_{47C55551-E54E-40CD-A718-3CAE99F89ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95672569-80AD-4ADF-9A80-EFA32C806D72}"/>
+  <xr:revisionPtr revIDLastSave="178" documentId="8_{47C55551-E54E-40CD-A718-3CAE99F89ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{381A6CBD-5B9E-4FA6-94FF-BC80D496E2F6}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FC573CD4-0E63-4713-BCBE-D8AF6B5A970C}"/>
+    <workbookView xWindow="3225" yWindow="1140" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{FC573CD4-0E63-4713-BCBE-D8AF6B5A970C}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
     <sheet name="Blad2" sheetId="2" r:id="rId2"/>
+    <sheet name="Blad3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="43">
   <si>
     <t>Thu</t>
   </si>
@@ -104,13 +105,73 @@
   </si>
   <si>
     <t>TOT</t>
+  </si>
+  <si>
+    <t>Måndag</t>
+  </si>
+  <si>
+    <t>Onsdag</t>
+  </si>
+  <si>
+    <t>Torsdag</t>
+  </si>
+  <si>
+    <t>Fredag</t>
+  </si>
+  <si>
+    <t>Kommentar</t>
+  </si>
+  <si>
+    <t>Idag</t>
+  </si>
+  <si>
+    <t>Onsdag förra veckan</t>
+  </si>
+  <si>
+    <t>Torsdag förra veckan</t>
+  </si>
+  <si>
+    <t>Fredag förra veckan</t>
+  </si>
+  <si>
+    <t>Lördag förra veckan</t>
+  </si>
+  <si>
+    <t>Söndag förra veckan</t>
+  </si>
+  <si>
+    <t>Igår</t>
+  </si>
+  <si>
+    <t>Förbrukning senaste veckan</t>
+  </si>
+  <si>
+    <t>imorgon onsdag kommer det fungerar på detta sätt</t>
+  </si>
+  <si>
+    <t>(om jag inte gör något mer idag)</t>
+  </si>
+  <si>
+    <t>Summa senaste veckan:</t>
+  </si>
+  <si>
+    <t>igår</t>
+  </si>
+  <si>
+    <t>i förrgår</t>
+  </si>
+  <si>
+    <t>morgondagens vecka</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -175,6 +236,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -197,7 +266,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -215,6 +284,7 @@
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlänk" xfId="1" builtinId="8"/>
@@ -936,4 +1006,205 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A970F86F-068A-496A-AD37-CE907E4A8548}">
+  <dimension ref="E4:P16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="4" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="K4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="K5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="5:16" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="E7" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="L7" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="I8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="F9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H9" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" t="s">
+        <v>34</v>
+      </c>
+      <c r="M9" t="s">
+        <v>23</v>
+      </c>
+      <c r="O9" t="s">
+        <v>20</v>
+      </c>
+      <c r="P9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="F10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10" s="1">
+        <v>9.0399999999999991</v>
+      </c>
+      <c r="H10" t="s">
+        <v>20</v>
+      </c>
+      <c r="I10" t="s">
+        <v>28</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="N10" s="1">
+        <v>9.0399999999999991</v>
+      </c>
+      <c r="O10" t="s">
+        <v>20</v>
+      </c>
+      <c r="P10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="F11" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" t="s">
+        <v>29</v>
+      </c>
+      <c r="M11" t="s">
+        <v>24</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="O11" t="s">
+        <v>20</v>
+      </c>
+      <c r="P11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="F12" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" t="s">
+        <v>20</v>
+      </c>
+      <c r="I12" t="s">
+        <v>30</v>
+      </c>
+      <c r="M12" t="s">
+        <v>25</v>
+      </c>
+      <c r="O12" t="s">
+        <v>20</v>
+      </c>
+      <c r="P12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="F13" t="s">
+        <v>26</v>
+      </c>
+      <c r="H13" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" t="s">
+        <v>31</v>
+      </c>
+      <c r="M13" t="s">
+        <v>26</v>
+      </c>
+      <c r="O13" t="s">
+        <v>20</v>
+      </c>
+      <c r="P13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="F14" t="s">
+        <v>6</v>
+      </c>
+      <c r="H14" t="s">
+        <v>20</v>
+      </c>
+      <c r="I14" t="s">
+        <v>32</v>
+      </c>
+      <c r="M14" t="s">
+        <v>6</v>
+      </c>
+      <c r="O14" t="s">
+        <v>20</v>
+      </c>
+      <c r="P14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="F15" t="s">
+        <v>7</v>
+      </c>
+      <c r="H15" t="s">
+        <v>20</v>
+      </c>
+      <c r="I15" t="s">
+        <v>33</v>
+      </c>
+      <c r="M15" t="s">
+        <v>7</v>
+      </c>
+      <c r="O15" t="s">
+        <v>20</v>
+      </c>
+      <c r="P15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="5:16" x14ac:dyDescent="0.25">
+      <c r="F16" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G16" s="1"/>
+      <c r="H16" t="s">
+        <v>20</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N16" s="1"/>
+      <c r="O16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>